<commit_message>
BWI sync — 2026-09-21 15:42 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Austria.xlsx
+++ b/BWI/bestwine_output/bestwine_Austria.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA886"/>
+  <dimension ref="A1:AA889"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -87769,6 +87769,317 @@
       <c r="Z886" s="2" t="inlineStr"/>
       <c r="AA886" s="2" t="inlineStr"/>
     </row>
+    <row r="887">
+      <c r="A887" s="2" t="inlineStr">
+        <is>
+          <t>Wedl Handels-gmbh</t>
+        </is>
+      </c>
+      <c r="B887" s="2" t="inlineStr">
+        <is>
+          <t>Wedl Handels-gmbh</t>
+        </is>
+      </c>
+      <c r="C887" s="2" t="inlineStr">
+        <is>
+          <t>105225</t>
+        </is>
+      </c>
+      <c r="D887" s="2" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E887" s="2" t="inlineStr">
+        <is>
+          <t>Mils</t>
+        </is>
+      </c>
+      <c r="F887" s="2" t="inlineStr">
+        <is>
+          <t>Tyrol</t>
+        </is>
+      </c>
+      <c r="G887" s="2" t="inlineStr">
+        <is>
+          <t>1 Leopold-Wedl-Straße</t>
+        </is>
+      </c>
+      <c r="H887" s="2" t="inlineStr">
+        <is>
+          <t>6068</t>
+        </is>
+      </c>
+      <c r="I887" s="2" t="inlineStr">
+        <is>
+          <t>https://www.wedl.com</t>
+        </is>
+      </c>
+      <c r="J887" s="2" t="inlineStr"/>
+      <c r="K887" s="2" t="inlineStr"/>
+      <c r="L887" s="2" t="inlineStr">
+        <is>
+          <t>2300</t>
+        </is>
+      </c>
+      <c r="M887" s="2" t="inlineStr"/>
+      <c r="N887" s="2" t="inlineStr">
+        <is>
+          <t>info@wedl.com</t>
+        </is>
+      </c>
+      <c r="O887" s="2" t="inlineStr">
+        <is>
+          <t>+43 59 3350</t>
+        </is>
+      </c>
+      <c r="P887" s="2" t="inlineStr">
+        <is>
+          <t>1978</t>
+        </is>
+      </c>
+      <c r="Q887" s="2" t="inlineStr">
+        <is>
+          <t>FN314555g</t>
+        </is>
+      </c>
+      <c r="R887" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/handelshauswedl/</t>
+        </is>
+      </c>
+      <c r="S887" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/handelshaus.wedl/</t>
+        </is>
+      </c>
+      <c r="T887" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/handelshaus.wedl/</t>
+        </is>
+      </c>
+      <c r="U887" s="2" t="inlineStr"/>
+      <c r="V887" s="2" t="inlineStr"/>
+      <c r="W887" s="2" t="inlineStr">
+        <is>
+          <t>Neubauer Manuela</t>
+        </is>
+      </c>
+      <c r="X887" s="2" t="inlineStr">
+        <is>
+          <t>Purchasing Manager, Central Purchasing</t>
+        </is>
+      </c>
+      <c r="Y887" s="2" t="inlineStr"/>
+      <c r="Z887" s="2" t="inlineStr"/>
+      <c r="AA887" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/neubauer-manuela-28837896/</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" s="2" t="inlineStr">
+        <is>
+          <t>Wedl Handels-gmbh</t>
+        </is>
+      </c>
+      <c r="B888" s="2" t="inlineStr">
+        <is>
+          <t>Wedl Handels-gmbh</t>
+        </is>
+      </c>
+      <c r="C888" s="2" t="inlineStr">
+        <is>
+          <t>105225</t>
+        </is>
+      </c>
+      <c r="D888" s="2" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E888" s="2" t="inlineStr">
+        <is>
+          <t>Mils</t>
+        </is>
+      </c>
+      <c r="F888" s="2" t="inlineStr">
+        <is>
+          <t>Tyrol</t>
+        </is>
+      </c>
+      <c r="G888" s="2" t="inlineStr">
+        <is>
+          <t>1 Leopold-Wedl-Straße</t>
+        </is>
+      </c>
+      <c r="H888" s="2" t="inlineStr">
+        <is>
+          <t>6068</t>
+        </is>
+      </c>
+      <c r="I888" s="2" t="inlineStr">
+        <is>
+          <t>https://www.wedl.com</t>
+        </is>
+      </c>
+      <c r="J888" s="2" t="inlineStr"/>
+      <c r="K888" s="2" t="inlineStr"/>
+      <c r="L888" s="2" t="inlineStr">
+        <is>
+          <t>2300</t>
+        </is>
+      </c>
+      <c r="M888" s="2" t="inlineStr"/>
+      <c r="N888" s="2" t="inlineStr">
+        <is>
+          <t>info@wedl.com</t>
+        </is>
+      </c>
+      <c r="O888" s="2" t="inlineStr">
+        <is>
+          <t>+43 59 3350</t>
+        </is>
+      </c>
+      <c r="P888" s="2" t="inlineStr">
+        <is>
+          <t>1978</t>
+        </is>
+      </c>
+      <c r="Q888" s="2" t="inlineStr">
+        <is>
+          <t>FN314555g</t>
+        </is>
+      </c>
+      <c r="R888" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/handelshauswedl/</t>
+        </is>
+      </c>
+      <c r="S888" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/handelshaus.wedl/</t>
+        </is>
+      </c>
+      <c r="T888" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/handelshaus.wedl/</t>
+        </is>
+      </c>
+      <c r="U888" s="2" t="inlineStr"/>
+      <c r="V888" s="2" t="inlineStr"/>
+      <c r="W888" s="2" t="inlineStr">
+        <is>
+          <t>Klaus Mantl</t>
+        </is>
+      </c>
+      <c r="X888" s="2" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="Y888" s="2" t="inlineStr"/>
+      <c r="Z888" s="2" t="inlineStr"/>
+      <c r="AA888" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/klaus-mantl-b0033a292/</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" s="2" t="inlineStr">
+        <is>
+          <t>Wine-world</t>
+        </is>
+      </c>
+      <c r="B889" s="2" t="inlineStr">
+        <is>
+          <t>Wine-world</t>
+        </is>
+      </c>
+      <c r="C889" s="2" t="inlineStr">
+        <is>
+          <t>89544</t>
+        </is>
+      </c>
+      <c r="D889" s="2" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
+      <c r="E889" s="2" t="inlineStr">
+        <is>
+          <t>Wien</t>
+        </is>
+      </c>
+      <c r="F889" s="2" t="inlineStr">
+        <is>
+          <t>Wien</t>
+        </is>
+      </c>
+      <c r="G889" s="2" t="inlineStr">
+        <is>
+          <t>124 Laxenburger Straße</t>
+        </is>
+      </c>
+      <c r="H889" s="2" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="I889" s="2" t="inlineStr">
+        <is>
+          <t>https://wine-world.at</t>
+        </is>
+      </c>
+      <c r="J889" s="2" t="inlineStr"/>
+      <c r="K889" s="2" t="inlineStr"/>
+      <c r="L889" s="2" t="inlineStr"/>
+      <c r="M889" s="2" t="inlineStr"/>
+      <c r="N889" s="2" t="inlineStr">
+        <is>
+          <t>orders@wine-world.at</t>
+        </is>
+      </c>
+      <c r="O889" s="2" t="inlineStr"/>
+      <c r="P889" s="2" t="inlineStr"/>
+      <c r="Q889" s="2" t="inlineStr"/>
+      <c r="R889" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/wine-world-at/</t>
+        </is>
+      </c>
+      <c r="S889" s="2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/wineworldnew</t>
+        </is>
+      </c>
+      <c r="T889" s="2" t="inlineStr"/>
+      <c r="U889" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/wineworldnew</t>
+        </is>
+      </c>
+      <c r="V889" s="2" t="inlineStr"/>
+      <c r="W889" s="2" t="inlineStr">
+        <is>
+          <t>Katharina Monsberger</t>
+        </is>
+      </c>
+      <c r="X889" s="2" t="inlineStr">
+        <is>
+          <t>Head of Sales</t>
+        </is>
+      </c>
+      <c r="Y889" s="2" t="inlineStr"/>
+      <c r="Z889" s="2" t="inlineStr"/>
+      <c r="AA889" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/katharina-monsberger-bb7bb11a1/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>